<commit_message>
WS2 integration: merge WS1 contacts into vendors.json, unify vendor ids, Drive anchors
- vendors.json now carries verified contacts, terms, public-price-page
  evidence, alias/active handling for duplicate + uncertain branches
- config/drive.json records the live Quick Entry Google Sheet id and the
  read-only Expense Tracker id
- ARCHITECTURE.md D2 amended with text-only Drive publishing mechanics
  (binary base64 uploads proved unreliable; entry sheet created from CSV)
- workbook regenerated from merged config; round-trip tests pass

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013xYzSQyKENNM7zVh34Euqx
</commit_message>
<xml_diff>
--- a/afuvai-price-monitor/AFUVAI Vendor Price Monitor.xlsx
+++ b/afuvai-price-monitor/AFUVAI Vendor Price Monitor.xlsx
@@ -1496,7 +1496,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LV Floral Wholesale</t>
+          <t>LV Floral Wholesale (Las Vegas Floral Wholesale)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1509,13 +1509,45 @@
           <t>lv-floral-wholesale</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>info@lvfloral.com</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>(702) 383-0603</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://www.lvfloral.com/</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2310 Highland Drive, Suite 140, Las Vegas, NV 89102</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Ask for new-account rep in outreach reply.</t>
+        </is>
+      </c>
+      <c r="T3" t="b">
+        <v>0</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>lvfloral.com</t>
+        </is>
+      </c>
       <c r="W3" t="b">
         <v>1</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Primary basis for AFUVAI bulk-tier pricing per spec.</t>
+          <t>Primary basis for AFUVAI bulk-tier pricing per spec. Hours Mon-Fri 7am-4pm, Sat 8am-12pm. Wholesale-only: registration form + resale certificate, 1-3 day review. Outreach draft r-6746775826887093567.</t>
         </is>
       </c>
     </row>
@@ -1537,18 +1569,46 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>las-vegas-floral-plant-wholesale</t>
-        </is>
+          <t>lv-floral-wholesale</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>info@lvfloral.com</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>(702) 383-0603</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://www.lvfloral.com/</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2310 Highland Drive, Suite 140, Las Vegas, NV 89102</t>
+        </is>
+      </c>
+      <c r="T4" t="b">
+        <v>0</v>
       </c>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>SAME COMPANY as lv-floral-wholesale (identical address/phone/site/email; Facebook page cross-match). Kept only because the spec lists it separately. Never log quotes under this id.</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>floral-supply-syndicate-las-vegas</t>
+          <t>fss-las-vegas</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1566,15 +1626,47 @@
           <t>floral-supply-syndicate</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>(702) 222-0453</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://www.fss.com/locations/las_vegas.php</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2861 S Highland Dr, Las Vegas, NV 89109</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Contact form: fss.com/contact.php; toll-free (800) 347-9994.</t>
+        </is>
+      </c>
+      <c r="T5" t="b">
+        <v>0</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>fss.com</t>
+        </is>
+      </c>
       <c r="W5" t="b">
         <v>1</v>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>HARD-GOODS wholesaler (packaging, ribbon, vases) — likely cannot quote fresh stems; keep for supplies cost tracking. Phone/contact-form outreach path.</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>floral-supply-syndicate-sparks</t>
+          <t>fss-sparks</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1591,16 +1683,39 @@
         <is>
           <t>floral-supply-syndicate</t>
         </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>(775) 331-2955</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://www.fss.com/reno</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>255 Greg St, Ste A, Sparks, NV 89431</t>
+        </is>
+      </c>
+      <c r="T6" t="b">
+        <v>0</v>
       </c>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Branch existence uncertain: Yelp (Jun 2026) marks it CLOSED while fss.com still lists it. Inactive until phone-verified.</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>greenleaf-wholesale-sparks</t>
+          <t>greenleaf-sparks</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1618,15 +1733,47 @@
           <t>greenleaf-wholesale</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>(775) 356-3700</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://www.greenleafwholesale.com/</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>255 Greg St, Ste B, Sparks, NV 89431</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>No verified email — LeadIQ shows only a format pattern; do NOT guess. Phone outreach.</t>
+        </is>
+      </c>
+      <c r="T7" t="b">
+        <v>0</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>greenleafwholesale.com</t>
+        </is>
+      </c>
       <c r="W7" t="b">
         <v>1</v>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Address moved from 605 Glendale Ave to 255 Greg St Ste B (per newer Yelp).</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>greenleaf-wholesale-hayward</t>
+          <t>greenleaf-hayward</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1643,16 +1790,44 @@
         <is>
           <t>greenleaf-wholesale</t>
         </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>(510) 471-2200</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://www.greenleafwholesale.com/</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1201 San Luis Obispo St, Hayward, CA 94544</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Directory (D&amp;B) lists contact 'Dave Kitayama' — unverified.</t>
+        </is>
+      </c>
+      <c r="T8" t="b">
+        <v>0</v>
       </c>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="b">
         <v>1</v>
       </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Older Tripaldi Way location marked CLOSED. Out-of-state: confirm they ship/deliver to Las Vegas before treating as a real option.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>san-diego-florist-supplies-lv</t>
+          <t>sdfs-las-vegas</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1670,9 +1845,51 @@
           <t>san-diego-florist-supplies</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>genew@sdfsinc.com</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>(702) 893-8080</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://www.sdfsinc.com/lasvegas</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>3950 W. Diablo Dr, Ste B-13, Las Vegas, NV 89118</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Gene W. (LV branch contact)</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Email published on company's own LV page.</t>
+        </is>
+      </c>
+      <c r="T9" t="b">
+        <v>0</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>sdfsinc.com</t>
+        </is>
+      </c>
       <c r="W9" t="b">
         <v>1</v>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Same Trade Center building as Mayesh. Outreach draft r-556253340011898982.</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1696,8 +1913,28 @@
           <t>las-vegas-flower-market</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>lasvegasflowermarket@gmail.com</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>(702) 873-8806</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://lasvegasflowermarket.com/</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Two LV stores; street addresses to confirm on first contact</t>
+        </is>
+      </c>
       <c r="L10" t="n">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -1709,20 +1946,37 @@
           <t>10:00-15:00</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Own vehicles, $18.95 fee</t>
+        </is>
+      </c>
+      <c r="T10" t="b">
+        <v>1</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>https://lasvegasflowermarket.com/shop-now</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>lasvegasflowermarket.com</t>
+        </is>
+      </c>
       <c r="W10" t="b">
         <v>1</v>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>Known facts from spec: $250 minimum order; delivery Mon-Sat 10am-3pm.</t>
+          <t>Spec said $250 minimum; current FAQ says $300 for wholesale/bulk (verifier-confirmed Jul 2026) — draft asks them to confirm. No account needed. Candidate for the optional portal-check path. Outreach draft r6454379485306042995. Email is gmail.com — also match full address in Gmail queries.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>mayesh-wholesale-las-vegas</t>
+          <t>mayesh-las-vegas</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1740,15 +1994,52 @@
           <t>mayesh-wholesale</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>tmetzger@mayesh.com</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>(702) 739-0418</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://www.mayesh.com/nv-las-vegas</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>3950 W Diablo Dr, Ste B-11, Las Vegas, NV 89118</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>tmetzger@ is LOW CONFIDENCE (possibly former manager; current mgr listed as Jacob Hunt). Phone-verify before sending draft r2959010547382611173.</t>
+        </is>
+      </c>
+      <c r="T11" t="b">
+        <v>0</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>mayesh.com</t>
+        </is>
+      </c>
       <c r="W11" t="b">
         <v>1</v>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>Resale license (or EIN) required to register; registered customers get a dedicated rep. Hours Mon-Thu 7am-3pm, Fri 7am-1pm.</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>floral-supply-syndicate-santa-ana-upland</t>
+          <t>fss-santa-ana-upland</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1765,6 +2056,24 @@
         <is>
           <t>floral-supply-syndicate</t>
         </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Santa Ana (714) 541-1233; Upland (909) 946-7226</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://www.fss.com/locations/santa_ana.php</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1605 E McFadden Ave, Santa Ana, CA 92705 / 2075 W Arrow Rte, Upland, CA 91786</t>
+        </is>
+      </c>
+      <c r="T12" t="b">
+        <v>0</v>
       </c>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="b">
@@ -1772,7 +2081,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>Backup branch — use when NV branches cannot fulfill.</t>
+          <t>Backup branches — out of state; same hard-goods caveat as fss-las-vegas. Covered by the FSS phone/contact-form outreach.</t>
         </is>
       </c>
     </row>

</xml_diff>